<commit_message>
20250501 第 7 次提交
</commit_message>
<xml_diff>
--- a/InfoSummary.xlsx
+++ b/InfoSummary.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="18408" firstSheet="2" activeTab="9"/>
+    <workbookView windowWidth="29868" windowHeight="14088" firstSheet="2"/>
   </bookViews>
   <sheets>
     <sheet name="学位" sheetId="10" r:id="rId1"/>
@@ -6217,7 +6217,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.77777777777778" style="1" customWidth="1"/>
@@ -6671,6 +6671,18 @@
         <v>1305</v>
       </c>
       <c r="J14" s="6"/>
+    </row>
+    <row r="15" customFormat="1" spans="1:10">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J14" etc:filterBottomFollowUsedRange="0">

</xml_diff>